<commit_message>
1단계 수집 결과 (phase1, 2026-10-24 23:05 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증계산" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원천값 확인" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="커버리지" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="안내" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="검증계산" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="원천값 확인" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="커버리지" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-25 02:42 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확인 표본" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증계산" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원천값 확인" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="커버리지" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="안내" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="확인 표본" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="검증계산" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="원천값 확인" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="커버리지" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1394591165007700</v>
+        <v>1388102989437300</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.1073211825482729</v>
+        <v>0.1078228158421242</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.4051830774339375</v>
+        <v>0.4070769563208435</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1227046858007700</v>
+        <v>1220558682437300</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.1458501196038896</v>
+        <v>0.1466254212723553</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>932838750105000</v>
+        <v>893392162395000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1736263528737086</v>
+        <v>0.1812926023055813</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2812711306969897</v>
+        <v>0.2936902975470612</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>904718344105000</v>
+        <v>865271756395000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.1422606890184407</v>
+        <v>0.1487461644838957</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>69561457610500</v>
+        <v>70947272762300</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.1171135177416166</v>
+        <v>0.1148259359777525</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.758560001501968</v>
+        <v>1.724209997611109</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>233986201610500</v>
+        <v>235372016762300</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.0410204487868796</v>
+        <v>0.04077893001908189</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26406103651200</v>
+        <v>26832008548800</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.07663145697601025</v>
+        <v>0.07541508464305771</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.118664247109649</v>
+        <v>1.100907671758702</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>22899366441858</v>
+        <v>23325271339458</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09796558634043065</v>
+        <v>0.09617679587315479</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>16962348197300</v>
+        <v>17635324785400</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.08915693643411493</v>
+        <v>-0.08575464406825202</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.088757204361578</v>
+        <v>2.009048737754584</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>46164934197300</v>
+        <v>46837910785400</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.01768327008787862</v>
+        <v>0.01742919328191867</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13267865274500</v>
+        <v>13445065478500</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.02610981217919059</v>
+        <v>0.02576569603844343</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.8880275724460138</v>
+        <v>0.8763237494154239</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6478646933917</v>
+        <v>6655847137917</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.1434132346578193</v>
+        <v>0.1395951099456555</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15156208333500</v>
+        <v>15446785460000</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.05000749417812824</v>
+        <v>0.04906677845449923</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.047728384110497</v>
+        <v>2.009207551976966</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12613182333500</v>
+        <v>12903759460000</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.07484637699184339</v>
+        <v>0.07316092669941943</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>33750008246500</v>
+        <v>33459997434500</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>9344993000000</v>
@@ -10992,7 +10992,7 @@
         <v/>
       </c>
       <c r="BA9" t="n">
-        <v>0.2383954380465784</v>
+        <v>0.2404617040318142</v>
       </c>
       <c r="BB9">
         <f>IF(AND(AZ9="",BA9=""),"",IF(OR(AZ9="",BA9=""),"불일치",IF(ABS(AZ9-BA9)&lt;=MAX(1,ABS(BA9))*1E-9,"일치","불일치")))</f>
@@ -11003,7 +11003,7 @@
         <v/>
       </c>
       <c r="BD9" t="n">
-        <v>1.102072027015201</v>
+        <v>1.111624113923242</v>
       </c>
       <c r="BE9">
         <f>IF(AND(BC9="",BD9=""),"",IF(OR(BC9="",BD9=""),"불일치",IF(ABS(BC9-BD9)&lt;=MAX(1,ABS(BD9))*1E-9,"일치","불일치")))</f>
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="BM9" t="n">
-        <v>78506441246500</v>
+        <v>78216430434500</v>
       </c>
       <c r="BN9">
         <f>IF(AND(BL9="",BM9=""),"",IF(OR(BL9="",BM9=""),"불일치",IF(ABS(BL9-BM9)&lt;=MAX(1,ABS(BM9))*1E-9,"일치","불일치")))</f>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="BP9" t="n">
-        <v>0.1239835463874621</v>
+        <v>0.1244432524717557</v>
       </c>
       <c r="BQ9">
         <f>IF(AND(BO9="",BP9=""),"",IF(OR(BO9="",BP9=""),"불일치",IF(ABS(BO9-BP9)&lt;=MAX(1,ABS(BP9))*1E-9,"일치","불일치")))</f>
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>23542850889</v>
+        <v>24241748074</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>716755534</v>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="BA10" t="n">
-        <v>-0.08117435921462332</v>
+        <v>-0.07883407702968773</v>
       </c>
       <c r="BB10">
         <f>IF(AND(AZ10="",BA10=""),"",IF(OR(AZ10="",BA10=""),"불일치",IF(ABS(AZ10-BA10)&lt;=MAX(1,ABS(BA10))*1E-9,"일치","불일치")))</f>
@@ -11255,7 +11255,7 @@
         <v/>
       </c>
       <c r="BD10" t="n">
-        <v>2.051379054886049</v>
+        <v>1.992237154621624</v>
       </c>
       <c r="BE10">
         <f>IF(AND(BC10="",BD10=""),"",IF(OR(BC10="",BD10=""),"불일치",IF(ABS(BC10-BD10)&lt;=MAX(1,ABS(BD10))*1E-9,"일치","불일치")))</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="BM10" t="n">
-        <v>99333796512</v>
+        <v>100032693697</v>
       </c>
       <c r="BN10">
         <f>IF(AND(BL10="",BM10=""),"",IF(OR(BL10="",BM10=""),"불일치",IF(ABS(BL10-BM10)&lt;=MAX(1,ABS(BM10))*1E-9,"일치","불일치")))</f>
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="BP10" t="n">
-        <v>0.00767001135316478</v>
+        <v>0.00761642337961803</v>
       </c>
       <c r="BQ10">
         <f>IF(AND(BO10="",BP10=""),"",IF(OR(BO10="",BP10=""),"불일치",IF(ABS(BO10-BP10)&lt;=MAX(1,ABS(BP10))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>125806444050</v>
+        <v>126238768600</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.1384777076369484</v>
+        <v>0.1380034689121643</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.6711390123580876</v>
+        <v>0.6688405910828886</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>61330000771</v>
+        <v>61762325321</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3398083503506891</v>
+        <v>0.3374297564200351</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>51308550810</v>
+        <v>53640757665</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4444493345845096</v>
+        <v>0.4251254504721396</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.160463321591133</v>
+        <v>3.023051872826301</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>125758466862</v>
+        <v>128090673717</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.03013952746544895</v>
+        <v>0.02959076298071619</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2181111967750</v>
+        <v>2211454182200</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.1836395600809935</v>
+        <v>-0.1811199370391369</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>2.932246218167128</v>
+        <v>2.892014390491043</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9591111803187</v>
+        <v>9621454017637</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.02651829969769367</v>
+        <v>0.0264346715958702</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>29085019200</v>
+        <v>29408186080</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-1542948785</v>
@@ -12735,7 +12735,7 @@
         <v/>
       </c>
       <c r="BA16" t="n">
-        <v>-0.2158556538274522</v>
+        <v>-0.2134836136755021</v>
       </c>
       <c r="BB16">
         <f>IF(AND(AZ16="",BA16=""),"",IF(OR(AZ16="",BA16=""),"불일치",IF(ABS(AZ16-BA16)&lt;=MAX(1,ABS(BA16))*1E-9,"일치","불일치")))</f>
@@ -12746,7 +12746,7 @@
         <v/>
       </c>
       <c r="BD16" t="n">
-        <v>1.748748642118827</v>
+        <v>1.729531624073565</v>
       </c>
       <c r="BE16">
         <f>IF(AND(BC16="",BD16=""),"",IF(OR(BC16="",BD16=""),"불일치",IF(ABS(BC16-BD16)&lt;=MAX(1,ABS(BD16))*1E-9,"일치","불일치")))</f>
@@ -12779,7 +12779,7 @@
         <v/>
       </c>
       <c r="BM16" t="n">
-        <v>28436332275</v>
+        <v>28759499155</v>
       </c>
       <c r="BN16">
         <f>IF(AND(BL16="",BM16=""),"",IF(OR(BL16="",BM16=""),"불일치",IF(ABS(BL16-BM16)&lt;=MAX(1,ABS(BM16))*1E-9,"일치","불일치")))</f>
@@ -12790,7 +12790,7 @@
         <v/>
       </c>
       <c r="BP16" t="n">
-        <v>-0.0720742360575754</v>
+        <v>-0.07126434691904843</v>
       </c>
       <c r="BQ16">
         <f>IF(AND(BO16="",BP16=""),"",IF(OR(BO16="",BP16=""),"불일치",IF(ABS(BO16-BP16)&lt;=MAX(1,ABS(BP16))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>19672900000</v>
+        <v>20940800000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.09397253190937788</v>
+        <v>0.08828278876642726</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.48749355641517</v>
+        <v>2.336883594991595</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>12280695291</v>
+        <v>13548595291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.0832328296386521</v>
+        <v>-0.07544376350801428</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>40178177708</v>
+        <v>40786499072</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.948715726905909</v>
+        <v>-1.919651074729045</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.834451725801501</v>
+        <v>4.762346977050201</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>207701260763</v>
+        <v>208309582127</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.2779954392423497</v>
+        <v>-0.2771836159788256</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>54903147400</v>
+        <v>55608325440</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8411939285105539</v>
+        <v>-0.8305266141997316</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.600100985886285</v>
+        <v>6.516404053094249</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>661882027159</v>
+        <v>662587205199</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.08827054306305401</v>
+        <v>0.08817659852555236</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>21063788130</v>
+        <v>21761021535</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1549987617540663</v>
+        <v>-0.1500325282408669</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.477927115572445</v>
+        <v>1.430573632948707</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28193606828</v>
+        <v>28890840233</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.1372958960737054</v>
+        <v>-0.1339824830909064</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>80288279220</v>
+        <v>84768388780</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02518045422869632</v>
+        <v>-0.02384963745443977</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.5765807337600578</v>
+        <v>0.5461077603485387</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>112907056108</v>
+        <v>117387165668</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.01428369179564262</v>
+        <v>0.0137385512447008</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>36092571570</v>
+        <v>36265263300</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.02623292436128291</v>
+        <v>-0.02610800567384823</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.5346262628191</v>
+        <v>1.527318518710438</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>34503111151</v>
+        <v>34675802881</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04642247236749772</v>
+        <v>-0.04619128011243928</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>488715915600</v>
+        <v>510739594200</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03219686668006684</v>
+        <v>0.03080850076573131</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.6347798075393802</v>
+        <v>0.607407372306676</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>552146496900</v>
+        <v>574170175500</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.02795025894331632</v>
+        <v>0.02687815951004582</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>104647861920</v>
+        <v>109794478080</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.1803237028715015</v>
+        <v>-0.1718710292993999</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.667451838322279</v>
+        <v>2.542415033400922</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>152046814298</v>
+        <v>157193430458</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2885043194001139</v>
+        <v>0.2790584984893529</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>21246412150</v>
+        <v>20909512520</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.0270412067196955</v>
+        <v>0.02747690183836003</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.095540709446324</v>
+        <v>2.12930461900601</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>43205605562</v>
+        <v>42868705932</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02847881338532135</v>
+        <v>0.02870262470604498</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-25 02:55 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="안내" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="확인 표본" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="검증계산" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="원천값 확인" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="커버리지" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확인 표본" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검증계산" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원천값 확인" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="커버리지" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45224,19 +45224,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="C11" t="n">
         <v>25</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>수정주가 미검증 25</t>
+          <t>가격 이력 부족(13개월 미만) 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-25 11:53 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1388102989437300</v>
+        <v>1394591165007700</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.1078228158421242</v>
+        <v>0.1073211825482729</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.4070769563208435</v>
+        <v>0.4051830774339375</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1220558682437300</v>
+        <v>1227046858007700</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.1466254212723553</v>
+        <v>0.1458501196038896</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>893392162395000</v>
+        <v>932838750105000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1812926023055813</v>
+        <v>0.1736263528737086</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2936902975470612</v>
+        <v>0.2812711306969897</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>865271756395000</v>
+        <v>904718344105000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.1487461644838957</v>
+        <v>0.1422606890184407</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>70947272762300</v>
+        <v>69561457610500</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.1148259359777525</v>
+        <v>0.1171135177416166</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.724209997611109</v>
+        <v>1.758560001501968</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>235372016762300</v>
+        <v>233986201610500</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.04077893001908189</v>
+        <v>0.0410204487868796</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26832008548800</v>
+        <v>26406103651200</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.07541508464305771</v>
+        <v>0.07663145697601025</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.100907671758702</v>
+        <v>1.118664247109649</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>23325271339458</v>
+        <v>22899366441858</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09617679587315479</v>
+        <v>0.09796558634043065</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>17635324785400</v>
+        <v>16962348197300</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.08575464406825202</v>
+        <v>-0.08915693643411493</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.009048737754584</v>
+        <v>2.088757204361578</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>46837910785400</v>
+        <v>46164934197300</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.01742919328191867</v>
+        <v>0.01768327008787862</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13445065478500</v>
+        <v>13267865274500</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.02576569603844343</v>
+        <v>0.02610981217919059</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.8763237494154239</v>
+        <v>0.8880275724460138</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6655847137917</v>
+        <v>6478646933917</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.1395951099456555</v>
+        <v>0.1434132346578193</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15446785460000</v>
+        <v>15156208333500</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.04906677845449923</v>
+        <v>0.05000749417812824</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.009207551976966</v>
+        <v>2.047728384110497</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12903759460000</v>
+        <v>12613182333500</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.07316092669941943</v>
+        <v>0.07484637699184339</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>33459997434500</v>
+        <v>33750008246500</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>9344993000000</v>
@@ -10992,7 +10992,7 @@
         <v/>
       </c>
       <c r="BA9" t="n">
-        <v>0.2404617040318142</v>
+        <v>0.2383954380465784</v>
       </c>
       <c r="BB9">
         <f>IF(AND(AZ9="",BA9=""),"",IF(OR(AZ9="",BA9=""),"불일치",IF(ABS(AZ9-BA9)&lt;=MAX(1,ABS(BA9))*1E-9,"일치","불일치")))</f>
@@ -11003,7 +11003,7 @@
         <v/>
       </c>
       <c r="BD9" t="n">
-        <v>1.111624113923242</v>
+        <v>1.102072027015201</v>
       </c>
       <c r="BE9">
         <f>IF(AND(BC9="",BD9=""),"",IF(OR(BC9="",BD9=""),"불일치",IF(ABS(BC9-BD9)&lt;=MAX(1,ABS(BD9))*1E-9,"일치","불일치")))</f>
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="BM9" t="n">
-        <v>78216430434500</v>
+        <v>78506441246500</v>
       </c>
       <c r="BN9">
         <f>IF(AND(BL9="",BM9=""),"",IF(OR(BL9="",BM9=""),"불일치",IF(ABS(BL9-BM9)&lt;=MAX(1,ABS(BM9))*1E-9,"일치","불일치")))</f>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="BP9" t="n">
-        <v>0.1244432524717557</v>
+        <v>0.1239835463874621</v>
       </c>
       <c r="BQ9">
         <f>IF(AND(BO9="",BP9=""),"",IF(OR(BO9="",BP9=""),"불일치",IF(ABS(BO9-BP9)&lt;=MAX(1,ABS(BP9))*1E-9,"일치","불일치")))</f>
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>24241748074</v>
+        <v>23542850889</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>716755534</v>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="BA10" t="n">
-        <v>-0.07883407702968773</v>
+        <v>-0.08117435921462332</v>
       </c>
       <c r="BB10">
         <f>IF(AND(AZ10="",BA10=""),"",IF(OR(AZ10="",BA10=""),"불일치",IF(ABS(AZ10-BA10)&lt;=MAX(1,ABS(BA10))*1E-9,"일치","불일치")))</f>
@@ -11255,7 +11255,7 @@
         <v/>
       </c>
       <c r="BD10" t="n">
-        <v>1.992237154621624</v>
+        <v>2.051379054886049</v>
       </c>
       <c r="BE10">
         <f>IF(AND(BC10="",BD10=""),"",IF(OR(BC10="",BD10=""),"불일치",IF(ABS(BC10-BD10)&lt;=MAX(1,ABS(BD10))*1E-9,"일치","불일치")))</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="BM10" t="n">
-        <v>100032693697</v>
+        <v>99333796512</v>
       </c>
       <c r="BN10">
         <f>IF(AND(BL10="",BM10=""),"",IF(OR(BL10="",BM10=""),"불일치",IF(ABS(BL10-BM10)&lt;=MAX(1,ABS(BM10))*1E-9,"일치","불일치")))</f>
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="BP10" t="n">
-        <v>0.00761642337961803</v>
+        <v>0.00767001135316478</v>
       </c>
       <c r="BQ10">
         <f>IF(AND(BO10="",BP10=""),"",IF(OR(BO10="",BP10=""),"불일치",IF(ABS(BO10-BP10)&lt;=MAX(1,ABS(BP10))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>126238768600</v>
+        <v>125806444050</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.1380034689121643</v>
+        <v>0.1384777076369484</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.6688405910828886</v>
+        <v>0.6711390123580876</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>61762325321</v>
+        <v>61330000771</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3374297564200351</v>
+        <v>0.3398083503506891</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>53640757665</v>
+        <v>51308550810</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4251254504721396</v>
+        <v>0.4444493345845096</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.023051872826301</v>
+        <v>3.160463321591133</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>128090673717</v>
+        <v>125758466862</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.02959076298071619</v>
+        <v>0.03013952746544895</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2211454182200</v>
+        <v>2181111967750</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.1811199370391369</v>
+        <v>-0.1836395600809935</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>2.892014390491043</v>
+        <v>2.932246218167128</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9621454017637</v>
+        <v>9591111803187</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.0264346715958702</v>
+        <v>0.02651829969769367</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>29408186080</v>
+        <v>29085019200</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-1542948785</v>
@@ -12735,7 +12735,7 @@
         <v/>
       </c>
       <c r="BA16" t="n">
-        <v>-0.2134836136755021</v>
+        <v>-0.2158556538274522</v>
       </c>
       <c r="BB16">
         <f>IF(AND(AZ16="",BA16=""),"",IF(OR(AZ16="",BA16=""),"불일치",IF(ABS(AZ16-BA16)&lt;=MAX(1,ABS(BA16))*1E-9,"일치","불일치")))</f>
@@ -12746,7 +12746,7 @@
         <v/>
       </c>
       <c r="BD16" t="n">
-        <v>1.729531624073565</v>
+        <v>1.748748642118827</v>
       </c>
       <c r="BE16">
         <f>IF(AND(BC16="",BD16=""),"",IF(OR(BC16="",BD16=""),"불일치",IF(ABS(BC16-BD16)&lt;=MAX(1,ABS(BD16))*1E-9,"일치","불일치")))</f>
@@ -12779,7 +12779,7 @@
         <v/>
       </c>
       <c r="BM16" t="n">
-        <v>28759499155</v>
+        <v>28436332275</v>
       </c>
       <c r="BN16">
         <f>IF(AND(BL16="",BM16=""),"",IF(OR(BL16="",BM16=""),"불일치",IF(ABS(BL16-BM16)&lt;=MAX(1,ABS(BM16))*1E-9,"일치","불일치")))</f>
@@ -12790,7 +12790,7 @@
         <v/>
       </c>
       <c r="BP16" t="n">
-        <v>-0.07126434691904843</v>
+        <v>-0.0720742360575754</v>
       </c>
       <c r="BQ16">
         <f>IF(AND(BO16="",BP16=""),"",IF(OR(BO16="",BP16=""),"불일치",IF(ABS(BO16-BP16)&lt;=MAX(1,ABS(BP16))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>20940800000</v>
+        <v>19672900000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.08828278876642726</v>
+        <v>0.09397253190937788</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.336883594991595</v>
+        <v>2.48749355641517</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>13548595291</v>
+        <v>12280695291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.07544376350801428</v>
+        <v>-0.0832328296386521</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>40786499072</v>
+        <v>40178177708</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.919651074729045</v>
+        <v>-1.948715726905909</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.762346977050201</v>
+        <v>4.834451725801501</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>208309582127</v>
+        <v>207701260763</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.2771836159788256</v>
+        <v>-0.2779954392423497</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>55608325440</v>
+        <v>54903147400</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8305266141997316</v>
+        <v>-0.8411939285105539</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.516404053094249</v>
+        <v>6.600100985886285</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>662587205199</v>
+        <v>661882027159</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.08817659852555236</v>
+        <v>0.08827054306305401</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>21761021535</v>
+        <v>21063788130</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1500325282408669</v>
+        <v>-0.1549987617540663</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.430573632948707</v>
+        <v>1.477927115572445</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28890840233</v>
+        <v>28193606828</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.1339824830909064</v>
+        <v>-0.1372958960737054</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>84768388780</v>
+        <v>80288279220</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02384963745443977</v>
+        <v>-0.02518045422869632</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.5461077603485387</v>
+        <v>0.5765807337600578</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>117387165668</v>
+        <v>112907056108</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.0137385512447008</v>
+        <v>0.01428369179564262</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>36265263300</v>
+        <v>36092571570</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.02610800567384823</v>
+        <v>-0.02623292436128291</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.527318518710438</v>
+        <v>1.5346262628191</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>34675802881</v>
+        <v>34503111151</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04619128011243928</v>
+        <v>-0.04642247236749772</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>510739594200</v>
+        <v>488715915600</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03080850076573131</v>
+        <v>0.03219686668006684</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.607407372306676</v>
+        <v>0.6347798075393802</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>574170175500</v>
+        <v>552146496900</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.02687815951004582</v>
+        <v>0.02795025894331632</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>109794478080</v>
+        <v>104647861920</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.1718710292993999</v>
+        <v>-0.1803237028715015</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.542415033400922</v>
+        <v>2.667451838322279</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>157193430458</v>
+        <v>152046814298</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2790584984893529</v>
+        <v>0.2885043194001139</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20909512520</v>
+        <v>21246412150</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.02747690183836003</v>
+        <v>0.0270412067196955</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.12930461900601</v>
+        <v>2.095540709446324</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>42868705932</v>
+        <v>43205605562</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02870262470604498</v>
+        <v>0.02847881338532135</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-27 10:34 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1394591165007700</v>
+        <v>1377006695036600</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.1073211825482729</v>
+        <v>0.1086916814126469</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.4051830774339375</v>
+        <v>0.4103572931321012</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1227046858007700</v>
+        <v>1209462388036600</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.1458501196038896</v>
+        <v>0.1479706461070902</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>932838750105000</v>
+        <v>931377765375000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1736263528737086</v>
+        <v>0.1738987079370399</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2812711306969897</v>
+        <v>0.2817123403137693</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>904718344105000</v>
+        <v>903257359375000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.1422606890184407</v>
+        <v>0.1424907903203321</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>69561457610500</v>
+        <v>67723117653200</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.1171135177416166</v>
+        <v>0.1202925571400516</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.758560001501968</v>
+        <v>1.806296007021169</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>233986201610500</v>
+        <v>232147861653200</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.0410204487868796</v>
+        <v>0.04134528283675748</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26406103651200</v>
+        <v>26497368986400</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.07663145697601025</v>
+        <v>0.07636751395542697</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.118664247109649</v>
+        <v>1.114811212963462</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>22899366441858</v>
+        <v>22990631777058</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09796558634043065</v>
+        <v>0.09757669480573407</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>16962348197300</v>
+        <v>16679210557400</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.08915693643411493</v>
+        <v>-0.09067041841072261</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.088757204361578</v>
+        <v>2.124214864850472</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>46164934197300</v>
+        <v>45881796557400</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.01768327008787862</v>
+        <v>0.01779239396126777</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13267865274500</v>
+        <v>13090665070500</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.02610981217919059</v>
+        <v>0.0264632444929529</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.8880275724460138</v>
+        <v>0.9000482502456215</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6478646933917</v>
+        <v>6301446729917</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.1434132346578193</v>
+        <v>0.1474460949717872</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15156208333500</v>
+        <v>15123560973500</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.05000749417812824</v>
+        <v>0.05011544578211833</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.047728384110497</v>
+        <v>2.05214883282991</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12613182333500</v>
+        <v>12580534973500</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.07484637699184339</v>
+        <v>0.07504060852647174</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>23542850889</v>
+        <v>23043638614</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>716755534</v>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="BA10" t="n">
-        <v>-0.08117435921462332</v>
+        <v>-0.08293290252516543</v>
       </c>
       <c r="BB10">
         <f>IF(AND(AZ10="",BA10=""),"",IF(OR(AZ10="",BA10=""),"불일치",IF(ABS(AZ10-BA10)&lt;=MAX(1,ABS(BA10))*1E-9,"일치","불일치")))</f>
@@ -11255,7 +11255,7 @@
         <v/>
       </c>
       <c r="BD10" t="n">
-        <v>2.051379054886049</v>
+        <v>2.095819675659144</v>
       </c>
       <c r="BE10">
         <f>IF(AND(BC10="",BD10=""),"",IF(OR(BC10="",BD10=""),"불일치",IF(ABS(BC10-BD10)&lt;=MAX(1,ABS(BD10))*1E-9,"일치","불일치")))</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="BM10" t="n">
-        <v>99333796512</v>
+        <v>98834584237</v>
       </c>
       <c r="BN10">
         <f>IF(AND(BL10="",BM10=""),"",IF(OR(BL10="",BM10=""),"불일치",IF(ABS(BL10-BM10)&lt;=MAX(1,ABS(BM10))*1E-9,"일치","불일치")))</f>
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="BP10" t="n">
-        <v>0.00767001135316478</v>
+        <v>0.007708752486609603</v>
       </c>
       <c r="BQ10">
         <f>IF(AND(BO10="",BP10=""),"",IF(OR(BO10="",BP10=""),"불일치",IF(ABS(BO10-BP10)&lt;=MAX(1,ABS(BP10))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>125806444050</v>
+        <v>125157957225</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.1384777076369484</v>
+        <v>0.1391952087127875</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.6711390123580876</v>
+        <v>0.6746164165671968</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>61330000771</v>
+        <v>60681513946</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3398083503506891</v>
+        <v>0.3434397897116698</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>51308550810</v>
+        <v>49753746240</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4444493345845096</v>
+        <v>0.4583383762902755</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.160463321591133</v>
+        <v>3.259227800390855</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>125758466862</v>
+        <v>124203662292</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.03013952746544895</v>
+        <v>0.03051681968192764</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2181111967750</v>
+        <v>2121192861700</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.1836395600809935</v>
+        <v>-0.1888269800813841</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>2.932246218167128</v>
+        <v>3.015075825641036</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9591111803187</v>
+        <v>9531192697137</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.02651829969769367</v>
+        <v>0.02668501050318699</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>29085019200</v>
+        <v>27792351680</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-1542948785</v>
@@ -12735,7 +12735,7 @@
         <v/>
       </c>
       <c r="BA16" t="n">
-        <v>-0.2158556538274522</v>
+        <v>-0.2258954516798918</v>
       </c>
       <c r="BB16">
         <f>IF(AND(AZ16="",BA16=""),"",IF(OR(AZ16="",BA16=""),"불일치",IF(ABS(AZ16-BA16)&lt;=MAX(1,ABS(BA16))*1E-9,"일치","불일치")))</f>
@@ -12746,7 +12746,7 @@
         <v/>
       </c>
       <c r="BD16" t="n">
-        <v>1.748748642118827</v>
+        <v>1.830085788263888</v>
       </c>
       <c r="BE16">
         <f>IF(AND(BC16="",BD16=""),"",IF(OR(BC16="",BD16=""),"불일치",IF(ABS(BC16-BD16)&lt;=MAX(1,ABS(BD16))*1E-9,"일치","불일치")))</f>
@@ -12779,7 +12779,7 @@
         <v/>
       </c>
       <c r="BM16" t="n">
-        <v>28436332275</v>
+        <v>27143664755</v>
       </c>
       <c r="BN16">
         <f>IF(AND(BL16="",BM16=""),"",IF(OR(BL16="",BM16=""),"불일치",IF(ABS(BL16-BM16)&lt;=MAX(1,ABS(BM16))*1E-9,"일치","불일치")))</f>
@@ -12790,7 +12790,7 @@
         <v/>
       </c>
       <c r="BP16" t="n">
-        <v>-0.0720742360575754</v>
+        <v>-0.07550664007602241</v>
       </c>
       <c r="BQ16">
         <f>IF(AND(BO16="",BP16=""),"",IF(OR(BO16="",BP16=""),"불일치",IF(ABS(BO16-BP16)&lt;=MAX(1,ABS(BP16))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>19672900000</v>
+        <v>19550200000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.09397253190937788</v>
+        <v>0.09456231767449949</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.48749355641517</v>
+        <v>2.503105440660454</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>12280695291</v>
+        <v>12157995291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.0832328296386521</v>
+        <v>-0.08407282570315316</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>40178177708</v>
+        <v>39946436236</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.948715726905909</v>
+        <v>-1.960020821768307</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.834451725801501</v>
+        <v>4.862497856190488</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>207701260763</v>
+        <v>207469519291</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.2779954392423497</v>
+        <v>-0.27830595749351</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>54903147400</v>
+        <v>54449818660</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8411939285105539</v>
+        <v>-0.8481973932252578</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.600100985886285</v>
+        <v>6.655050947840935</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>661882027159</v>
+        <v>661428698419</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.08827054306305401</v>
+        <v>0.0883310417595296</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>21063788130</v>
+        <v>20917002150</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1549987617540663</v>
+        <v>-0.1560864723628668</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.477927115572445</v>
+        <v>1.488298533927339</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28193606828</v>
+        <v>28046820848</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.1372958960737054</v>
+        <v>-0.1380144485529464</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>80288279220</v>
+        <v>73921807740</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02518045422869632</v>
+        <v>-0.02734910578906251</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.5765807337600578</v>
+        <v>0.6262384046102063</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>112907056108</v>
+        <v>106540584628</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.01428369179564262</v>
+        <v>0.01513723241364829</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>36092571570</v>
+        <v>35919879840</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.02623292436128291</v>
+        <v>-0.02635904418994292</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.5346262628191</v>
+        <v>1.542004273698038</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>34503111151</v>
+        <v>34330419421</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04642247236749772</v>
+        <v>-0.04665599054756157</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>488715915600</v>
+        <v>468789730200</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03219686668006684</v>
+        <v>0.03356541358593098</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.6347798075393802</v>
+        <v>0.6617614995824411</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>552146496900</v>
+        <v>532220311500</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.02795025894331632</v>
+        <v>0.02899670912503308</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>104647861920</v>
+        <v>101431226820</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.1803237028715015</v>
+        <v>-0.1860422135333885</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.667451838322279</v>
+        <v>2.752043334252161</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>152046814298</v>
+        <v>148830179198</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2885043194001139</v>
+        <v>0.2947397020710533</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>21246412150</v>
+        <v>20963851170</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.0270412067196955</v>
+        <v>0.02740568125298325</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.095540709446324</v>
+        <v>2.123785426110712</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>43205605562</v>
+        <v>42923044582</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02847881338532135</v>
+        <v>0.02866628847004001</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-28 10:35 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1377006695036600</v>
+        <v>1435159563809300</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.1086916814126469</v>
+        <v>0.1042874790889019</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.4103572931321012</v>
+        <v>0.3937295574996316</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1209462388036600</v>
+        <v>1267615256809300</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.1479706461070902</v>
+        <v>0.1411823737830914</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>931377765375000</v>
+        <v>979590261465000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1738987079370399</v>
+        <v>0.1653399348394675</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2817123403137693</v>
+        <v>0.2678473034303176</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>903257359375000</v>
+        <v>951469855465000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.1424907903203321</v>
+        <v>0.1352705545643369</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>67723117653200</v>
+        <v>68348529566400</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.1202925571400516</v>
+        <v>0.1191918399954115</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.806296007021169</v>
+        <v>1.789767794216544</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>232147861653200</v>
+        <v>232773273566400</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.04134528283675748</v>
+        <v>0.04123419692021494</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26497368986400</v>
+        <v>26512579875600</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.07636751395542697</v>
+        <v>0.07632370012068491</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.114811212963462</v>
+        <v>1.114171619611217</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>22990631777058</v>
+        <v>23005842666258</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09757669480573407</v>
+        <v>0.09751217952956168</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>16679210557400</v>
+        <v>16938576165300</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.09067041841072261</v>
+        <v>-0.08928206156418787</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.124214864850472</v>
+        <v>2.09168861976614</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>45881796557400</v>
+        <v>46141162165300</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.01779239396126777</v>
+        <v>0.01769238054896514</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13090665070500</v>
+        <v>13068515045000</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.0264632444929529</v>
+        <v>0.02650809744972062</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.9000482502456215</v>
+        <v>0.9015737557545124</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6301446729917</v>
+        <v>6279296704417</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.1474460949717872</v>
+        <v>0.1479662065252361</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15123560973500</v>
+        <v>15095430412000</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.05011544578211833</v>
+        <v>0.05020883666871095</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.05214883282991</v>
+        <v>2.05597304302952</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12580534973500</v>
+        <v>12552404412000</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.07504060852647174</v>
+        <v>0.07520877825586106</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>33750008246500</v>
+        <v>36070094742500</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>9344993000000</v>
@@ -10992,7 +10992,7 @@
         <v/>
       </c>
       <c r="BA9" t="n">
-        <v>0.2383954380465784</v>
+        <v>0.2230614601219743</v>
       </c>
       <c r="BB9">
         <f>IF(AND(AZ9="",BA9=""),"",IF(OR(AZ9="",BA9=""),"불일치",IF(ABS(AZ9-BA9)&lt;=MAX(1,ABS(BA9))*1E-9,"일치","불일치")))</f>
@@ -11003,7 +11003,7 @@
         <v/>
       </c>
       <c r="BD9" t="n">
-        <v>1.102072027015201</v>
+        <v>1.031184982061459</v>
       </c>
       <c r="BE9">
         <f>IF(AND(BC9="",BD9=""),"",IF(OR(BC9="",BD9=""),"불일치",IF(ABS(BC9-BD9)&lt;=MAX(1,ABS(BD9))*1E-9,"일치","불일치")))</f>
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="BM9" t="n">
-        <v>78506441246500</v>
+        <v>80826527742500</v>
       </c>
       <c r="BN9">
         <f>IF(AND(BL9="",BM9=""),"",IF(OR(BL9="",BM9=""),"불일치",IF(ABS(BL9-BM9)&lt;=MAX(1,ABS(BM9))*1E-9,"일치","불일치")))</f>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="BP9" t="n">
-        <v>0.1239835463874621</v>
+        <v>0.1204246584860029</v>
       </c>
       <c r="BQ9">
         <f>IF(AND(BO9="",BP9=""),"",IF(OR(BO9="",BP9=""),"불일치",IF(ABS(BO9-BP9)&lt;=MAX(1,ABS(BP9))*1E-9,"일치","불일치")))</f>
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>23043638614</v>
+        <v>23702598817</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>716755534</v>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="BA10" t="n">
-        <v>-0.08293290252516543</v>
+        <v>-0.08062727002025349</v>
       </c>
       <c r="BB10">
         <f>IF(AND(AZ10="",BA10=""),"",IF(OR(AZ10="",BA10=""),"불일치",IF(ABS(AZ10-BA10)&lt;=MAX(1,ABS(BA10))*1E-9,"일치","불일치")))</f>
@@ -11255,7 +11255,7 @@
         <v/>
       </c>
       <c r="BD10" t="n">
-        <v>2.095819675659144</v>
+        <v>2.037553416773927</v>
       </c>
       <c r="BE10">
         <f>IF(AND(BC10="",BD10=""),"",IF(OR(BC10="",BD10=""),"불일치",IF(ABS(BC10-BD10)&lt;=MAX(1,ABS(BD10))*1E-9,"일치","불일치")))</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="BM10" t="n">
-        <v>98834584237</v>
+        <v>99493544440</v>
       </c>
       <c r="BN10">
         <f>IF(AND(BL10="",BM10=""),"",IF(OR(BL10="",BM10=""),"불일치",IF(ABS(BL10-BM10)&lt;=MAX(1,ABS(BM10))*1E-9,"일치","불일치")))</f>
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="BP10" t="n">
-        <v>0.007708752486609603</v>
+        <v>0.007657696298672541</v>
       </c>
       <c r="BQ10">
         <f>IF(AND(BO10="",BP10=""),"",IF(OR(BO10="",BP10=""),"불일치",IF(ABS(BO10-BP10)&lt;=MAX(1,ABS(BP10))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>125157957225</v>
+        <v>124509470400</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.1391952087127875</v>
+        <v>0.1399201837581666</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.6746164165671968</v>
+        <v>0.6781300437368176</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>60681513946</v>
+        <v>60033027121</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3434397897116698</v>
+        <v>0.3471496839064085</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>49753746240</v>
+        <v>49400381565</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4583383762902755</v>
+        <v>0.4616169054482889</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.259227800390855</v>
+        <v>3.282541303970189</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>124203662292</v>
+        <v>123850297617</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.03051681968192764</v>
+        <v>0.0306038890412786</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2121192861700</v>
+        <v>2121112301400</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.1888269800813841</v>
+        <v>-0.1888341517705744</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>3.015075825641036</v>
+        <v>3.015190338867364</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9531192697137</v>
+        <v>9531112136837</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.02668501050318699</v>
+        <v>0.02668523605424764</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>27792351680</v>
+        <v>28681060600</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-1542948785</v>
@@ -12735,7 +12735,7 @@
         <v/>
       </c>
       <c r="BA16" t="n">
-        <v>-0.2258954516798918</v>
+        <v>-0.2188958743038952</v>
       </c>
       <c r="BB16">
         <f>IF(AND(AZ16="",BA16=""),"",IF(OR(AZ16="",BA16=""),"불일치",IF(ABS(AZ16-BA16)&lt;=MAX(1,ABS(BA16))*1E-9,"일치","불일치")))</f>
@@ -12746,7 +12746,7 @@
         <v/>
       </c>
       <c r="BD16" t="n">
-        <v>1.830085788263888</v>
+        <v>1.77337890468388</v>
       </c>
       <c r="BE16">
         <f>IF(AND(BC16="",BD16=""),"",IF(OR(BC16="",BD16=""),"불일치",IF(ABS(BC16-BD16)&lt;=MAX(1,ABS(BD16))*1E-9,"일치","불일치")))</f>
@@ -12779,7 +12779,7 @@
         <v/>
       </c>
       <c r="BM16" t="n">
-        <v>27143664755</v>
+        <v>28032373675</v>
       </c>
       <c r="BN16">
         <f>IF(AND(BL16="",BM16=""),"",IF(OR(BL16="",BM16=""),"불일치",IF(ABS(BL16-BM16)&lt;=MAX(1,ABS(BM16))*1E-9,"일치","불일치")))</f>
@@ -12790,7 +12790,7 @@
         <v/>
       </c>
       <c r="BP16" t="n">
-        <v>-0.07550664007602241</v>
+        <v>-0.07311285689758842</v>
       </c>
       <c r="BQ16">
         <f>IF(AND(BO16="",BP16=""),"",IF(OR(BO16="",BP16=""),"불일치",IF(ABS(BO16-BP16)&lt;=MAX(1,ABS(BP16))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>19550200000</v>
+        <v>19509300000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.09456231767449949</v>
+        <v>0.09476056152706658</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.503105440660454</v>
+        <v>2.508353041164983</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>12157995291</v>
+        <v>12117095291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.08407282570315316</v>
+        <v>-0.08435660481759266</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>39946436236</v>
+        <v>40178177708</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.960020821768307</v>
+        <v>-1.948715726905909</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.862497856190488</v>
+        <v>4.834451725801501</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>207469519291</v>
+        <v>207701260763</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.27830595749351</v>
+        <v>-0.2779954392423497</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>54449818660</v>
+        <v>55356476140</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8481973932252578</v>
+        <v>-0.8343051702242982</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.655050947840935</v>
+        <v>6.546051023308508</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>661428698419</v>
+        <v>662335355899</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.0883310417595296</v>
+        <v>0.08821012718202111</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>20917002150</v>
+        <v>21430753080</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1560864723628668</v>
+        <v>-0.1523446733678666</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.488298533927339</v>
+        <v>1.452620144415382</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28046820848</v>
+        <v>28560571778</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.1380144485529464</v>
+        <v>-0.1355318283922348</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>73921807740</v>
+        <v>77812429200</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02734910578906251</v>
+        <v>-0.02598165049960939</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.6262384046102063</v>
+        <v>0.594926484379696</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>106540584628</v>
+        <v>110431206088</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.01513723241364829</v>
+        <v>0.01460392988658346</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>35919879840</v>
+        <v>35056421190</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.02635904418994292</v>
+        <v>-0.02700828173156714</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.542004273698038</v>
+        <v>1.579984674528039</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>34330419421</v>
+        <v>33466960771</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04665599054756157</v>
+        <v>-0.04785973052527471</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>468789730200</v>
+        <v>479277196200</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03356541358593098</v>
+        <v>0.03283094064094343</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.6617614995824411</v>
+        <v>0.6472809416047072</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>532220311500</v>
+        <v>542707777500</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.02899670912503308</v>
+        <v>0.02843636705206422</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>101431226820</v>
+        <v>103146765540</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.1860422135333885</v>
+        <v>-0.182947956343644</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.752043334252161</v>
+        <v>2.706271303744848</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>148830179198</v>
+        <v>150545717918</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2947397020710533</v>
+        <v>0.2913810056018547</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20963851170</v>
+        <v>20985586630</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.02740568125298325</v>
+        <v>0.02737729629052547</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.123785426110712</v>
+        <v>2.121585751925201</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>42923044582</v>
+        <v>42944780042</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02866628847004001</v>
+        <v>0.02865177972262578</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-29 10:30 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1435159563809300</v>
+        <v>1567330188826300</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.1042874790889019</v>
+        <v>0.09549307099870272</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.3937295574996316</v>
+        <v>0.3605269291872381</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1267615256809300</v>
+        <v>1399785881826300</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.1411823737830914</v>
+        <v>0.12785164740089</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>979590261465000</v>
+        <v>1086242146755000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1653399348394675</v>
+        <v>0.1491061550906025</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2678473034303176</v>
+        <v>0.2415489131809387</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>951469855465000</v>
+        <v>1058121740755000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.1352705545643369</v>
+        <v>0.121636150211</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>68348529566400</v>
+        <v>69665687790800</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.1191918399954115</v>
+        <v>0.116938298584857</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.789767794216544</v>
+        <v>1.755928935451557</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>232773273566400</v>
+        <v>234090431790800</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.04123419692021494</v>
+        <v>0.04100218418400654</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26512579875600</v>
+        <v>27075382776000</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.07632370012068491</v>
+        <v>0.07473719624177179</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.114171619611217</v>
+        <v>1.091011872461995</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>23005842666258</v>
+        <v>23568645566658</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09751217952956168</v>
+        <v>0.09518365635209065</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>16938576165300</v>
+        <v>17484152516700</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.08928206156418787</v>
+        <v>-0.08649609974263923</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.09168861976614</v>
+        <v>2.026419465636598</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>46141162165300</v>
+        <v>46686738516700</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.01769238054896514</v>
+        <v>0.01748562923726167</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13068515045000</v>
+        <v>13201415198000</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.02650809744972062</v>
+        <v>0.02624123740828048</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.9015737557545124</v>
+        <v>0.8924975098912119</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6279296704417</v>
+        <v>6412196857417</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.1479662065252361</v>
+        <v>0.1448994367545471</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15095430412000</v>
+        <v>15278667536200</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.05020883666871095</v>
+        <v>0.04960668187878545</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.05597304302952</v>
+        <v>2.031315749653324</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12552404412000</v>
+        <v>12735641536200</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.07520877825586106</v>
+        <v>0.07412669376070406</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>36070094742500</v>
+        <v>39151459620000</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>9344993000000</v>
@@ -10992,7 +10992,7 @@
         <v/>
       </c>
       <c r="BA9" t="n">
-        <v>0.2230614601219743</v>
+        <v>0.205505697056819</v>
       </c>
       <c r="BB9">
         <f>IF(AND(AZ9="",BA9=""),"",IF(OR(AZ9="",BA9=""),"불일치",IF(ABS(AZ9-BA9)&lt;=MAX(1,ABS(BA9))*1E-9,"일치","불일치")))</f>
@@ -11003,7 +11003,7 @@
         <v/>
       </c>
       <c r="BD9" t="n">
-        <v>1.031184982061459</v>
+        <v>0.9500269047695852</v>
       </c>
       <c r="BE9">
         <f>IF(AND(BC9="",BD9=""),"",IF(OR(BC9="",BD9=""),"불일치",IF(ABS(BC9-BD9)&lt;=MAX(1,ABS(BD9))*1E-9,"일치","불일치")))</f>
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="BM9" t="n">
-        <v>80826527742500</v>
+        <v>83907892620000</v>
       </c>
       <c r="BN9">
         <f>IF(AND(BL9="",BM9=""),"",IF(OR(BL9="",BM9=""),"불일치",IF(ABS(BL9-BM9)&lt;=MAX(1,ABS(BM9))*1E-9,"일치","불일치")))</f>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="BP9" t="n">
-        <v>0.1204246584860029</v>
+        <v>0.1160022817410141</v>
       </c>
       <c r="BQ9">
         <f>IF(AND(BO9="",BP9=""),"",IF(OR(BO9="",BP9=""),"불일치",IF(ABS(BO9-BP9)&lt;=MAX(1,ABS(BP9))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>124509470400</v>
+        <v>122347847650</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.1399201837581666</v>
+        <v>0.142392271810431</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.6781300437368176</v>
+        <v>0.6901111399159133</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>60033027121</v>
+        <v>57871404371</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3471496839064085</v>
+        <v>0.3601164792096073</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>49400381565</v>
+        <v>49965765045</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4616169054482889</v>
+        <v>0.4563935175507128</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.282541303970189</v>
+        <v>3.245397979455675</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>123850297617</v>
+        <v>124415681097</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.0306038890412786</v>
+        <v>0.03046481546843692</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2121112301400</v>
+        <v>2150930873900</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.1888341517705744</v>
+        <v>-0.186216324803947</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>3.015190338867364</v>
+        <v>2.973390449892877</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9531112136837</v>
+        <v>9560930709337</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.02668523605424764</v>
+        <v>0.0266020103024716</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>28681060600</v>
+        <v>27994330980</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-1542948785</v>
@@ -12735,7 +12735,7 @@
         <v/>
       </c>
       <c r="BA16" t="n">
-        <v>-0.2188958743038952</v>
+        <v>-0.2242656143661841</v>
       </c>
       <c r="BB16">
         <f>IF(AND(AZ16="",BA16=""),"",IF(OR(AZ16="",BA16=""),"불일치",IF(ABS(AZ16-BA16)&lt;=MAX(1,ABS(BA16))*1E-9,"일치","불일치")))</f>
@@ -12746,7 +12746,7 @@
         <v/>
       </c>
       <c r="BD16" t="n">
-        <v>1.77337890468388</v>
+        <v>1.816881706097482</v>
       </c>
       <c r="BE16">
         <f>IF(AND(BC16="",BD16=""),"",IF(OR(BC16="",BD16=""),"불일치",IF(ABS(BC16-BD16)&lt;=MAX(1,ABS(BD16))*1E-9,"일치","불일치")))</f>
@@ -12779,7 +12779,7 @@
         <v/>
       </c>
       <c r="BM16" t="n">
-        <v>28032373675</v>
+        <v>27345644055</v>
       </c>
       <c r="BN16">
         <f>IF(AND(BL16="",BM16=""),"",IF(OR(BL16="",BM16=""),"불일치",IF(ABS(BL16-BM16)&lt;=MAX(1,ABS(BM16))*1E-9,"일치","불일치")))</f>
@@ -12790,7 +12790,7 @@
         <v/>
       </c>
       <c r="BP16" t="n">
-        <v>-0.07311285689758842</v>
+        <v>-0.07494893595769068</v>
       </c>
       <c r="BQ16">
         <f>IF(AND(BO16="",BP16=""),"",IF(OR(BO16="",BP16=""),"불일치",IF(ABS(BO16-BP16)&lt;=MAX(1,ABS(BP16))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>19509300000</v>
+        <v>20204600000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.09476056152706658</v>
+        <v>0.09149957054334161</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.508353041164983</v>
+        <v>2.422033199667402</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>12117095291</v>
+        <v>12812395291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.08435660481759266</v>
+        <v>-0.07977876078472297</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>40178177708</v>
+        <v>41930824394</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.948715726905909</v>
+        <v>-1.86726228042403</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.834451725801501</v>
+        <v>4.63237876591318</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>207701260763</v>
+        <v>209453907449</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.2779954392423497</v>
+        <v>-0.275669257834491</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>55356476140</v>
+        <v>54399448800</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8343051702242982</v>
+        <v>-0.8489827611819478</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.546051023308508</v>
+        <v>6.661213032051898</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>662335355899</v>
+        <v>661378328559</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.08821012718202111</v>
+        <v>0.08833776895637739</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>21430753080</v>
+        <v>21834414525</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1523446733678666</v>
+        <v>-0.1495282172215699</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.452620144415382</v>
+        <v>1.425764982081653</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28560571778</v>
+        <v>28964233223</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.1355318283922348</v>
+        <v>-0.133642982474199</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>77812429200</v>
+        <v>78637712540</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02598165049960939</v>
+        <v>-0.02570897950486086</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.594926484379696</v>
+        <v>0.5886828780968506</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>110431206088</v>
+        <v>111256489428</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.01460392988658346</v>
+        <v>0.01449560020535866</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>35056421190</v>
+        <v>34469269308</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.02700828173156714</v>
+        <v>-0.0274683426428263</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.579984674528039</v>
+        <v>1.606898241128216</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>33466960771</v>
+        <v>32879808889</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04785973052527471</v>
+        <v>-0.04871438667442676</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>479277196200</v>
+        <v>503398368000</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03283094064094343</v>
+        <v>0.03125779140189823</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.6472809416047072</v>
+        <v>0.6162653964861483</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>542707777500</v>
+        <v>566828949300</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.02843636705206422</v>
+        <v>0.02722626919824471</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>103146765540</v>
+        <v>104004534900</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.182947956343644</v>
+        <v>-0.1814391072191603</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.706271303744848</v>
+        <v>2.683951540414994</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>150545717918</v>
+        <v>151403487278</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2913810056018547</v>
+        <v>0.2897302001733619</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20985586630</v>
+        <v>20659554730</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.02737729629052547</v>
+        <v>0.02780934199737227</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.121585751925201</v>
+        <v>2.155066852692038</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>42944780042</v>
+        <v>42618748142</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02865177972262578</v>
+        <v>0.02887096481342725</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-10-31 04:17 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1567330188826300</v>
+        <v>1503892701287700</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.09549307099870272</v>
+        <v>0.09952117785520641</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.3605269291872381</v>
+        <v>0.3757347445839496</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1399785881826300</v>
+        <v>1336348394287700</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.12785164740089</v>
+        <v>0.1339208635749451</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1086242146755000</v>
+        <v>1114731348990000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1491061550906025</v>
+        <v>0.1452954473261638</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2415489131809387</v>
+        <v>0.2353756447575727</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>1058121740755000</v>
+        <v>1086610942990000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.121636150211</v>
+        <v>0.1184470447590407</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>69665687790800</v>
+        <v>68892569498300</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.116938298584857</v>
+        <v>0.1182505901482021</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.755928935451557</v>
+        <v>1.775634119772795</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>234090431790800</v>
+        <v>233317313498300</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.04100218418400654</v>
+        <v>0.0411380486775146</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>27075382776000</v>
+        <v>26603845210800</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.07473719624177179</v>
+        <v>0.0760618692454853</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.091011872461995</v>
+        <v>1.11034941851478</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>23568645566658</v>
+        <v>23097108001458</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09518365635209065</v>
+        <v>0.09712687234087442</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>17484152516700</v>
+        <v>17342967834700</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.08649609974263923</v>
+        <v>-0.08720024245066935</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.026419465636598</v>
+        <v>2.042916030156662</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>46686738516700</v>
+        <v>46545553834700</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.01748562923726167</v>
+        <v>0.0175386676652112</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13201415198000</v>
+        <v>12979914943000</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.02624123740828048</v>
+        <v>0.02668904009442861</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.8924975098912119</v>
+        <v>0.907727842824509</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6412196857417</v>
+        <v>6190696602417</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.1448994367545471</v>
+        <v>0.150083871439645</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15278667536200</v>
+        <v>15232707695200</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.04960668187878545</v>
+        <v>0.04975635423233589</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.031315749653324</v>
+        <v>2.0374445975734</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12735641536200</v>
+        <v>12689681695200</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.07412669376070406</v>
+        <v>0.0743951678754162</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>39151459620000</v>
+        <v>38788946105000</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>9344993000000</v>
@@ -10992,7 +10992,7 @@
         <v/>
       </c>
       <c r="BA9" t="n">
-        <v>0.205505697056819</v>
+        <v>0.2074263110480042</v>
       </c>
       <c r="BB9">
         <f>IF(AND(AZ9="",BA9=""),"",IF(OR(AZ9="",BA9=""),"불일치",IF(ABS(AZ9-BA9)&lt;=MAX(1,ABS(BA9))*1E-9,"일치","불일치")))</f>
@@ -11003,7 +11003,7 @@
         <v/>
       </c>
       <c r="BD9" t="n">
-        <v>0.9500269047695852</v>
+        <v>0.9589056608889271</v>
       </c>
       <c r="BE9">
         <f>IF(AND(BC9="",BD9=""),"",IF(OR(BC9="",BD9=""),"불일치",IF(ABS(BC9-BD9)&lt;=MAX(1,ABS(BD9))*1E-9,"일치","불일치")))</f>
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="BM9" t="n">
-        <v>83907892620000</v>
+        <v>83545379105000</v>
       </c>
       <c r="BN9">
         <f>IF(AND(BL9="",BM9=""),"",IF(OR(BL9="",BM9=""),"불일치",IF(ABS(BL9-BM9)&lt;=MAX(1,ABS(BM9))*1E-9,"일치","불일치")))</f>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="BP9" t="n">
-        <v>0.1160022817410141</v>
+        <v>0.1165056296861962</v>
       </c>
       <c r="BQ9">
         <f>IF(AND(BO9="",BP9=""),"",IF(OR(BO9="",BP9=""),"불일치",IF(ABS(BO9-BP9)&lt;=MAX(1,ABS(BP9))*1E-9,"일치","불일치")))</f>
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>23702598817</v>
+        <v>26238597174</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>716755534</v>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="BA10" t="n">
-        <v>-0.08062727002025349</v>
+        <v>-0.07283452778846339</v>
       </c>
       <c r="BB10">
         <f>IF(AND(AZ10="",BA10=""),"",IF(OR(AZ10="",BA10=""),"불일치",IF(ABS(AZ10-BA10)&lt;=MAX(1,ABS(BA10))*1E-9,"일치","불일치")))</f>
@@ -11255,7 +11255,7 @@
         <v/>
       </c>
       <c r="BD10" t="n">
-        <v>2.037553416773927</v>
+        <v>1.840620932808715</v>
       </c>
       <c r="BE10">
         <f>IF(AND(BC10="",BD10=""),"",IF(OR(BC10="",BD10=""),"불일치",IF(ABS(BC10-BD10)&lt;=MAX(1,ABS(BD10))*1E-9,"일치","불일치")))</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="BM10" t="n">
-        <v>99493544440</v>
+        <v>102029542797</v>
       </c>
       <c r="BN10">
         <f>IF(AND(BL10="",BM10=""),"",IF(OR(BL10="",BM10=""),"불일치",IF(ABS(BL10-BM10)&lt;=MAX(1,ABS(BM10))*1E-9,"일치","불일치")))</f>
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="BP10" t="n">
-        <v>0.007657696298672541</v>
+        <v>0.007467360198956043</v>
       </c>
       <c r="BQ10">
         <f>IF(AND(BO10="",BP10=""),"",IF(OR(BO10="",BP10=""),"불일치",IF(ABS(BO10-BP10)&lt;=MAX(1,ABS(BP10))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>122347847650</v>
+        <v>122564009925</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.142392271810431</v>
+        <v>0.1421411390559152</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.6901111399159133</v>
+        <v>0.688894012685021</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>57871404371</v>
+        <v>58087566646</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3601164792096073</v>
+        <v>0.3587763714738962</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>49965765045</v>
+        <v>48834998085</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4563935175507128</v>
+        <v>0.4669612400989203</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.245397979455675</v>
+        <v>3.320544676519772</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>124415681097</v>
+        <v>123284914137</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.03046481546843692</v>
+        <v>0.03074423819436691</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2150930873900</v>
+        <v>2160816691200</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.186216324803947</v>
+        <v>-0.1853643781428598</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>2.973390449892877</v>
+        <v>2.959787077210263</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9560930709337</v>
+        <v>9570816526637</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.0266020103024716</v>
+        <v>0.02657453274996278</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>20204600000</v>
+        <v>21104400000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.09149957054334161</v>
+        <v>0.08759842606281154</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.422033199667402</v>
+        <v>2.318768218286234</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>12812395291</v>
+        <v>13712195291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.07977876078472297</v>
+        <v>-0.07454364507708644</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>41930824394</v>
+        <v>41509711380</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.86726228042403</v>
+        <v>-1.886205520950071</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.63237876591318</v>
+        <v>4.679373912813749</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>209453907449</v>
+        <v>209032794435</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.275669257834491</v>
+        <v>-0.276224615247894</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>54399448800</v>
+        <v>53744640620</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8489827611819478</v>
+        <v>-0.8593265061635461</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.661213032051898</v>
+        <v>6.742371203951312</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>661378328559</v>
+        <v>660723520379</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.08833776895637739</v>
+        <v>0.088425315852971</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>21834414525</v>
+        <v>21430753080</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1495282172215699</v>
+        <v>-0.1523446733678666</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.425764982081653</v>
+        <v>1.452620144415382</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28964233223</v>
+        <v>28560571778</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.133642982474199</v>
+        <v>-0.1355318283922348</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>78637712540</v>
+        <v>73568114880</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02570897950486086</v>
+        <v>-0.02748059187458685</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.5886828780968506</v>
+        <v>0.6292491661708323</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>111256489428</v>
+        <v>106186891768</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.01449560020535866</v>
+        <v>0.01518765230009308</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>34469269308</v>
+        <v>34003001637</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.0274683426428263</v>
+        <v>-0.02784500351197627</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.606898241128216</v>
+        <v>1.628932904668319</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>32879808889</v>
+        <v>32413541218</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04871438667442676</v>
+        <v>-0.04941514144435806</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>503398368000</v>
+        <v>492910902000</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03125779140189823</v>
+        <v>0.03192285079342798</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.6162653964861483</v>
+        <v>0.6293774261986196</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>566828949300</v>
+        <v>556341483300</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.02722626919824471</v>
+        <v>0.027739505369004</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>104004534900</v>
+        <v>101645669160</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.1814391072191603</v>
+        <v>-0.18564971941201</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.683951540414994</v>
+        <v>2.746237335656692</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>151403487278</v>
+        <v>149044621538</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2897302001733619</v>
+        <v>0.2943156366418496</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20659554730</v>
+        <v>20474803320</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.02780934199737227</v>
+        <v>0.02806027555042712</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.155066852692038</v>
+        <v>2.17451278501463</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>42618748142</v>
+        <v>42433996732</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02887096481342725</v>
+        <v>0.02899666476790075</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>

<commit_message>
1단계 실행 결과 (phase1, 2026-11-01 10:47 KST)
</commit_message>
<xml_diff>
--- a/reports/phase1/verification_workbook.xlsx
+++ b/reports/phase1/verification_workbook.xlsx
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1503892701287700</v>
+        <v>1455105513242300</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>118370658000000</v>
@@ -9255,7 +9255,7 @@
         <v/>
       </c>
       <c r="BA2" t="n">
-        <v>0.09952117785520641</v>
+        <v>0.1028579519752514</v>
       </c>
       <c r="BB2">
         <f>IF(AND(AZ2="",BA2=""),"",IF(OR(AZ2="",BA2=""),"불일치",IF(ABS(AZ2-BA2)&lt;=MAX(1,ABS(BA2))*1E-9,"일치","불일치")))</f>
@@ -9266,7 +9266,7 @@
         <v/>
       </c>
       <c r="BD2" t="n">
-        <v>0.3757347445839496</v>
+        <v>0.3883324850724464</v>
       </c>
       <c r="BE2">
         <f>IF(AND(BC2="",BD2=""),"",IF(OR(BC2="",BD2=""),"불일치",IF(ABS(BC2-BD2)&lt;=MAX(1,ABS(BD2))*1E-9,"일치","불일치")))</f>
@@ -9299,7 +9299,7 @@
         <v/>
       </c>
       <c r="BM2" t="n">
-        <v>1336348394287700</v>
+        <v>1287561206242300</v>
       </c>
       <c r="BN2">
         <f>IF(AND(BL2="",BM2=""),"",IF(OR(BL2="",BM2=""),"불일치",IF(ABS(BL2-BM2)&lt;=MAX(1,ABS(BM2))*1E-9,"일치","불일치")))</f>
@@ -9310,7 +9310,7 @@
         <v/>
       </c>
       <c r="BP2" t="n">
-        <v>0.1339208635749451</v>
+        <v>0.1389952804824732</v>
       </c>
       <c r="BQ2">
         <f>IF(AND(BO2="",BP2=""),"",IF(OR(BO2="",BP2=""),"불일치",IF(ABS(BO2-BP2)&lt;=MAX(1,ABS(BP2))*1E-9,"일치","불일치")))</f>
@@ -9350,7 +9350,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1114731348990000</v>
+        <v>1035838173570000</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>134150412000000</v>
@@ -9507,7 +9507,7 @@
         <v/>
       </c>
       <c r="BA3" t="n">
-        <v>0.1452954473261638</v>
+        <v>0.1563616732156036</v>
       </c>
       <c r="BB3">
         <f>IF(AND(AZ3="",BA3=""),"",IF(OR(AZ3="",BA3=""),"불일치",IF(ABS(AZ3-BA3)&lt;=MAX(1,ABS(BA3))*1E-9,"일치","불일치")))</f>
@@ -9518,7 +9518,7 @@
         <v/>
       </c>
       <c r="BD3" t="n">
-        <v>0.2353756447575727</v>
+        <v>0.2533027037376981</v>
       </c>
       <c r="BE3">
         <f>IF(AND(BC3="",BD3=""),"",IF(OR(BC3="",BD3=""),"불일치",IF(ABS(BC3-BD3)&lt;=MAX(1,ABS(BD3))*1E-9,"일치","불일치")))</f>
@@ -9551,7 +9551,7 @@
         <v/>
       </c>
       <c r="BM3" t="n">
-        <v>1086610942990000</v>
+        <v>1007717767570000</v>
       </c>
       <c r="BN3">
         <f>IF(AND(BL3="",BM3=""),"",IF(OR(BL3="",BM3=""),"불일치",IF(ABS(BL3-BM3)&lt;=MAX(1,ABS(BM3))*1E-9,"일치","불일치")))</f>
@@ -9562,7 +9562,7 @@
         <v/>
       </c>
       <c r="BP3" t="n">
-        <v>0.1184470447590407</v>
+        <v>0.1277201406405287</v>
       </c>
       <c r="BQ3">
         <f>IF(AND(BO3="",BP3=""),"",IF(OR(BO3="",BP3=""),"불일치",IF(ABS(BO3-BP3)&lt;=MAX(1,ABS(BP3))*1E-9,"일치","불일치")))</f>
@@ -9602,7 +9602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>68892569498300</v>
+        <v>66270568998500</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>4856197000000</v>
@@ -9759,7 +9759,7 @@
         <v/>
       </c>
       <c r="BA4" t="n">
-        <v>0.1182505901482021</v>
+        <v>0.1229291844496521</v>
       </c>
       <c r="BB4">
         <f>IF(AND(AZ4="",BA4=""),"",IF(OR(AZ4="",BA4=""),"불일치",IF(ABS(AZ4-BA4)&lt;=MAX(1,ABS(BA4))*1E-9,"일치","불일치")))</f>
@@ -9770,7 +9770,7 @@
         <v/>
       </c>
       <c r="BD4" t="n">
-        <v>1.775634119772795</v>
+        <v>1.845887229409013</v>
       </c>
       <c r="BE4">
         <f>IF(AND(BC4="",BD4=""),"",IF(OR(BC4="",BD4=""),"불일치",IF(ABS(BC4-BD4)&lt;=MAX(1,ABS(BD4))*1E-9,"일치","불일치")))</f>
@@ -9803,7 +9803,7 @@
         <v/>
       </c>
       <c r="BM4" t="n">
-        <v>233317313498300</v>
+        <v>230695312998500</v>
       </c>
       <c r="BN4">
         <f>IF(AND(BL4="",BM4=""),"",IF(OR(BL4="",BM4=""),"불일치",IF(ABS(BL4-BM4)&lt;=MAX(1,ABS(BM4))*1E-9,"일치","불일치")))</f>
@@ -9814,7 +9814,7 @@
         <v/>
       </c>
       <c r="BP4" t="n">
-        <v>0.0411380486775146</v>
+        <v>0.04160560904010394</v>
       </c>
       <c r="BQ4">
         <f>IF(AND(BO4="",BP4=""),"",IF(OR(BO4="",BP4=""),"불일치",IF(ABS(BO4-BP4)&lt;=MAX(1,ABS(BP4))*1E-9,"일치","불일치")))</f>
@@ -9854,7 +9854,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>26603845210800</v>
+        <v>26208362091600</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>983946430695</v>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="BA5" t="n">
-        <v>0.0760618692454853</v>
+        <v>0.07720963976224829</v>
       </c>
       <c r="BB5">
         <f>IF(AND(AZ5="",BA5=""),"",IF(OR(AZ5="",BA5=""),"불일치",IF(ABS(AZ5-BA5)&lt;=MAX(1,ABS(BA5))*1E-9,"일치","불일치")))</f>
@@ -10013,7 +10013,7 @@
         <v/>
       </c>
       <c r="BD5" t="n">
-        <v>1.11034941851478</v>
+        <v>1.127104546130209</v>
       </c>
       <c r="BE5">
         <f>IF(AND(BC5="",BD5=""),"",IF(OR(BC5="",BD5=""),"불일치",IF(ABS(BC5-BD5)&lt;=MAX(1,ABS(BD5))*1E-9,"일치","불일치")))</f>
@@ -10043,7 +10043,7 @@
         <v/>
       </c>
       <c r="BM5" t="n">
-        <v>23097108001458</v>
+        <v>22701624882258</v>
       </c>
       <c r="BN5">
         <f>IF(AND(BL5="",BM5=""),"",IF(OR(BL5="",BM5=""),"불일치",IF(ABS(BL5-BM5)&lt;=MAX(1,ABS(BM5))*1E-9,"일치","불일치")))</f>
@@ -10054,7 +10054,7 @@
         <v/>
       </c>
       <c r="BP5" t="n">
-        <v>0.09712687234087442</v>
+        <v>0.09881891150682545</v>
       </c>
       <c r="BQ5">
         <f>IF(AND(BO5="",BP5=""),"",IF(OR(BO5="",BP5=""),"불일치",IF(ABS(BO5-BP5)&lt;=MAX(1,ABS(BP5))*1E-9,"일치","불일치")))</f>
@@ -10094,7 +10094,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>17342967834700</v>
+        <v>17388975346900</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>-234766000000</v>
@@ -10251,7 +10251,7 @@
         <v/>
       </c>
       <c r="BA6" t="n">
-        <v>-0.08720024245066935</v>
+        <v>-0.08696952924656401</v>
       </c>
       <c r="BB6">
         <f>IF(AND(AZ6="",BA6=""),"",IF(OR(AZ6="",BA6=""),"불일치",IF(ABS(AZ6-BA6)&lt;=MAX(1,ABS(BA6))*1E-9,"일치","불일치")))</f>
@@ -10262,7 +10262,7 @@
         <v/>
       </c>
       <c r="BD6" t="n">
-        <v>2.042916030156662</v>
+        <v>2.037510910975918</v>
       </c>
       <c r="BE6">
         <f>IF(AND(BC6="",BD6=""),"",IF(OR(BC6="",BD6=""),"불일치",IF(ABS(BC6-BD6)&lt;=MAX(1,ABS(BD6))*1E-9,"일치","불일치")))</f>
@@ -10295,7 +10295,7 @@
         <v/>
       </c>
       <c r="BM6" t="n">
-        <v>46545553834700</v>
+        <v>46591561346900</v>
       </c>
       <c r="BN6">
         <f>IF(AND(BL6="",BM6=""),"",IF(OR(BL6="",BM6=""),"불일치",IF(ABS(BL6-BM6)&lt;=MAX(1,ABS(BM6))*1E-9,"일치","불일치")))</f>
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="BP6" t="n">
-        <v>0.0175386676652112</v>
+        <v>0.01752134885375152</v>
       </c>
       <c r="BQ6">
         <f>IF(AND(BO6="",BP6=""),"",IF(OR(BO6="",BP6=""),"불일치",IF(ABS(BO6-BP6)&lt;=MAX(1,ABS(BP6))*1E-9,"일치","불일치")))</f>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>12979914943000</v>
+        <v>13046365019500</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>188028656200</v>
@@ -10491,7 +10491,7 @@
         <v/>
       </c>
       <c r="BA7" t="n">
-        <v>0.02668904009442861</v>
+        <v>0.02655310270854867</v>
       </c>
       <c r="BB7">
         <f>IF(AND(AZ7="",BA7=""),"",IF(OR(AZ7="",BA7=""),"불일치",IF(ABS(AZ7-BA7)&lt;=MAX(1,ABS(BA7))*1E-9,"일치","불일치")))</f>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="BD7" t="n">
-        <v>0.907727842824509</v>
+        <v>0.9031044412481533</v>
       </c>
       <c r="BE7">
         <f>IF(AND(BC7="",BD7=""),"",IF(OR(BC7="",BD7=""),"불일치",IF(ABS(BC7-BD7)&lt;=MAX(1,ABS(BD7))*1E-9,"일치","불일치")))</f>
@@ -10532,7 +10532,7 @@
         <v/>
       </c>
       <c r="BM7" t="n">
-        <v>6190696602417</v>
+        <v>6257146678917</v>
       </c>
       <c r="BN7">
         <f>IF(AND(BL7="",BM7=""),"",IF(OR(BL7="",BM7=""),"불일치",IF(ABS(BL7-BM7)&lt;=MAX(1,ABS(BM7))*1E-9,"일치","불일치")))</f>
@@ -10543,7 +10543,7 @@
         <v/>
       </c>
       <c r="BP7" t="n">
-        <v>0.150083871439645</v>
+        <v>0.1484900004229747</v>
       </c>
       <c r="BQ7">
         <f>IF(AND(BO7="",BP7=""),"",IF(OR(BO7="",BP7=""),"불일치",IF(ABS(BO7-BP7)&lt;=MAX(1,ABS(BP7))*1E-9,"일치","불일치")))</f>
@@ -10583,7 +10583,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>15232707695200</v>
+        <v>14730762883000</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>805510000000</v>
@@ -10740,7 +10740,7 @@
         <v/>
       </c>
       <c r="BA8" t="n">
-        <v>0.04975635423233589</v>
+        <v>0.05145178196267624</v>
       </c>
       <c r="BB8">
         <f>IF(AND(AZ8="",BA8=""),"",IF(OR(AZ8="",BA8=""),"불일치",IF(ABS(AZ8-BA8)&lt;=MAX(1,ABS(BA8))*1E-9,"일치","불일치")))</f>
@@ -10751,7 +10751,7 @@
         <v/>
       </c>
       <c r="BD8" t="n">
-        <v>2.0374445975734</v>
+        <v>2.106869701623993</v>
       </c>
       <c r="BE8">
         <f>IF(AND(BC8="",BD8=""),"",IF(OR(BC8="",BD8=""),"불일치",IF(ABS(BC8-BD8)&lt;=MAX(1,ABS(BD8))*1E-9,"일치","불일치")))</f>
@@ -10784,7 +10784,7 @@
         <v/>
       </c>
       <c r="BM8" t="n">
-        <v>12689681695200</v>
+        <v>12187736883000</v>
       </c>
       <c r="BN8">
         <f>IF(AND(BL8="",BM8=""),"",IF(OR(BL8="",BM8=""),"불일치",IF(ABS(BL8-BM8)&lt;=MAX(1,ABS(BM8))*1E-9,"일치","불일치")))</f>
@@ -10795,7 +10795,7 @@
         <v/>
       </c>
       <c r="BP8" t="n">
-        <v>0.0743951678754162</v>
+        <v>0.07745908933403416</v>
       </c>
       <c r="BQ8">
         <f>IF(AND(BO8="",BP8=""),"",IF(OR(BO8="",BP8=""),"불일치",IF(ABS(BO8-BP8)&lt;=MAX(1,ABS(BP8))*1E-9,"일치","불일치")))</f>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>38788946105000</v>
+        <v>36468859609000</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>9344993000000</v>
@@ -10992,7 +10992,7 @@
         <v/>
       </c>
       <c r="BA9" t="n">
-        <v>0.2074263110480042</v>
+        <v>0.2206224183114955</v>
       </c>
       <c r="BB9">
         <f>IF(AND(AZ9="",BA9=""),"",IF(OR(AZ9="",BA9=""),"불일치",IF(ABS(AZ9-BA9)&lt;=MAX(1,ABS(BA9))*1E-9,"일치","불일치")))</f>
@@ -11003,7 +11003,7 @@
         <v/>
       </c>
       <c r="BD9" t="n">
-        <v>0.9589056608889271</v>
+        <v>1.019909599553829</v>
       </c>
       <c r="BE9">
         <f>IF(AND(BC9="",BD9=""),"",IF(OR(BC9="",BD9=""),"불일치",IF(ABS(BC9-BD9)&lt;=MAX(1,ABS(BD9))*1E-9,"일치","불일치")))</f>
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="BM9" t="n">
-        <v>83545379105000</v>
+        <v>81225292609000</v>
       </c>
       <c r="BN9">
         <f>IF(AND(BL9="",BM9=""),"",IF(OR(BL9="",BM9=""),"불일치",IF(ABS(BL9-BM9)&lt;=MAX(1,ABS(BM9))*1E-9,"일치","불일치")))</f>
@@ -11047,7 +11047,7 @@
         <v/>
       </c>
       <c r="BP9" t="n">
-        <v>0.1165056296861962</v>
+        <v>0.1198334495002053</v>
       </c>
       <c r="BQ9">
         <f>IF(AND(BO9="",BP9=""),"",IF(OR(BO9="",BP9=""),"불일치",IF(ABS(BO9-BP9)&lt;=MAX(1,ABS(BP9))*1E-9,"일치","불일치")))</f>
@@ -11087,7 +11087,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>26238597174</v>
+        <v>23702598817</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>716755534</v>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="BA10" t="n">
-        <v>-0.07283452778846339</v>
+        <v>-0.08062727002025349</v>
       </c>
       <c r="BB10">
         <f>IF(AND(AZ10="",BA10=""),"",IF(OR(AZ10="",BA10=""),"불일치",IF(ABS(AZ10-BA10)&lt;=MAX(1,ABS(BA10))*1E-9,"일치","불일치")))</f>
@@ -11255,7 +11255,7 @@
         <v/>
       </c>
       <c r="BD10" t="n">
-        <v>1.840620932808715</v>
+        <v>2.037553416773927</v>
       </c>
       <c r="BE10">
         <f>IF(AND(BC10="",BD10=""),"",IF(OR(BC10="",BD10=""),"불일치",IF(ABS(BC10-BD10)&lt;=MAX(1,ABS(BD10))*1E-9,"일치","불일치")))</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="BM10" t="n">
-        <v>102029542797</v>
+        <v>99493544440</v>
       </c>
       <c r="BN10">
         <f>IF(AND(BL10="",BM10=""),"",IF(OR(BL10="",BM10=""),"불일치",IF(ABS(BL10-BM10)&lt;=MAX(1,ABS(BM10))*1E-9,"일치","불일치")))</f>
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="BP10" t="n">
-        <v>0.007467360198956043</v>
+        <v>0.007657696298672541</v>
       </c>
       <c r="BQ10">
         <f>IF(AND(BO10="",BP10=""),"",IF(OR(BO10="",BP10=""),"불일치",IF(ABS(BO10-BP10)&lt;=MAX(1,ABS(BP10))*1E-9,"일치","불일치")))</f>
@@ -11336,7 +11336,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>122564009925</v>
+        <v>124077145850</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>9977068365</v>
@@ -11493,7 +11493,7 @@
         <v/>
       </c>
       <c r="BA11" t="n">
-        <v>0.1421411390559152</v>
+        <v>0.1404077105308431</v>
       </c>
       <c r="BB11">
         <f>IF(AND(AZ11="",BA11=""),"",IF(OR(AZ11="",BA11=""),"불일치",IF(ABS(AZ11-BA11)&lt;=MAX(1,ABS(BA11))*1E-9,"일치","불일치")))</f>
@@ -11504,7 +11504,7 @@
         <v/>
       </c>
       <c r="BD11" t="n">
-        <v>0.688894012685021</v>
+        <v>0.6804928661888623</v>
       </c>
       <c r="BE11">
         <f>IF(AND(BC11="",BD11=""),"",IF(OR(BC11="",BD11=""),"불일치",IF(ABS(BC11-BD11)&lt;=MAX(1,ABS(BD11))*1E-9,"일치","불일치")))</f>
@@ -11537,7 +11537,7 @@
         <v/>
       </c>
       <c r="BM11" t="n">
-        <v>58087566646</v>
+        <v>59600702571</v>
       </c>
       <c r="BN11">
         <f>IF(AND(BL11="",BM11=""),"",IF(OR(BL11="",BM11=""),"불일치",IF(ABS(BL11-BM11)&lt;=MAX(1,ABS(BM11))*1E-9,"일치","불일치")))</f>
@@ -11548,7 +11548,7 @@
         <v/>
       </c>
       <c r="BP11" t="n">
-        <v>0.3587763714738962</v>
+        <v>0.3496677973581534</v>
       </c>
       <c r="BQ11">
         <f>IF(AND(BO11="",BP11=""),"",IF(OR(BO11="",BP11=""),"불일치",IF(ABS(BO11-BP11)&lt;=MAX(1,ABS(BP11))*1E-9,"일치","불일치")))</f>
@@ -11588,7 +11588,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>48834998085</v>
+        <v>48128268735</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>4468961675</v>
@@ -11745,7 +11745,7 @@
         <v/>
       </c>
       <c r="BA12" t="n">
-        <v>0.4669612400989203</v>
+        <v>0.4738182333456005</v>
       </c>
       <c r="BB12">
         <f>IF(AND(AZ12="",BA12=""),"",IF(OR(AZ12="",BA12=""),"불일치",IF(ABS(AZ12-BA12)&lt;=MAX(1,ABS(BA12))*1E-9,"일치","불일치")))</f>
@@ -11756,7 +11756,7 @@
         <v/>
       </c>
       <c r="BD12" t="n">
-        <v>3.320544676519772</v>
+        <v>3.369304510242529</v>
       </c>
       <c r="BE12">
         <f>IF(AND(BC12="",BD12=""),"",IF(OR(BC12="",BD12=""),"불일치",IF(ABS(BC12-BD12)&lt;=MAX(1,ABS(BD12))*1E-9,"일치","불일치")))</f>
@@ -11789,7 +11789,7 @@
         <v/>
       </c>
       <c r="BM12" t="n">
-        <v>123284914137</v>
+        <v>122578184787</v>
       </c>
       <c r="BN12">
         <f>IF(AND(BL12="",BM12=""),"",IF(OR(BL12="",BM12=""),"불일치",IF(ABS(BL12-BM12)&lt;=MAX(1,ABS(BM12))*1E-9,"일치","불일치")))</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="BP12" t="n">
-        <v>0.03074423819436691</v>
+        <v>0.0309214953100038</v>
       </c>
       <c r="BQ12">
         <f>IF(AND(BO12="",BP12=""),"",IF(OR(BO12="",BP12=""),"불일치",IF(ABS(BO12-BP12)&lt;=MAX(1,ABS(BP12))*1E-9,"일치","불일치")))</f>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2160816691200</v>
+        <v>2165799880000</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>42120798515</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="BA13" t="n">
-        <v>-0.1853643781428598</v>
+        <v>-0.1849378818162092</v>
       </c>
       <c r="BB13">
         <f>IF(AND(AZ13="",BA13=""),"",IF(OR(AZ13="",BA13=""),"불일치",IF(ABS(AZ13-BA13)&lt;=MAX(1,ABS(BA13))*1E-9,"일치","불일치")))</f>
@@ -12008,7 +12008,7 @@
         <v/>
       </c>
       <c r="BD13" t="n">
-        <v>2.959787077210263</v>
+        <v>2.952977039981183</v>
       </c>
       <c r="BE13">
         <f>IF(AND(BC13="",BD13=""),"",IF(OR(BC13="",BD13=""),"불일치",IF(ABS(BC13-BD13)&lt;=MAX(1,ABS(BD13))*1E-9,"일치","불일치")))</f>
@@ -12041,7 +12041,7 @@
         <v/>
       </c>
       <c r="BM13" t="n">
-        <v>9570816526637</v>
+        <v>9575799715437</v>
       </c>
       <c r="BN13">
         <f>IF(AND(BL13="",BM13=""),"",IF(OR(BL13="",BM13=""),"불일치",IF(ABS(BL13-BM13)&lt;=MAX(1,ABS(BM13))*1E-9,"일치","불일치")))</f>
@@ -12052,7 +12052,7 @@
         <v/>
       </c>
       <c r="BP13" t="n">
-        <v>0.02657453274996278</v>
+        <v>0.02656070352233688</v>
       </c>
       <c r="BQ13">
         <f>IF(AND(BO13="",BP13=""),"",IF(OR(BO13="",BP13=""),"불일치",IF(ABS(BO13-BP13)&lt;=MAX(1,ABS(BP13))*1E-9,"일치","불일치")))</f>
@@ -12578,7 +12578,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>27994330980</v>
+        <v>27711559960</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-1542948785</v>
@@ -12735,7 +12735,7 @@
         <v/>
       </c>
       <c r="BA16" t="n">
-        <v>-0.2242656143661841</v>
+        <v>-0.2265540390025737</v>
       </c>
       <c r="BB16">
         <f>IF(AND(AZ16="",BA16=""),"",IF(OR(AZ16="",BA16=""),"불일치",IF(ABS(AZ16-BA16)&lt;=MAX(1,ABS(BA16))*1E-9,"일치","불일치")))</f>
@@ -12746,7 +12746,7 @@
         <v/>
       </c>
       <c r="BD16" t="n">
-        <v>1.816881706097482</v>
+        <v>1.835421315343375</v>
       </c>
       <c r="BE16">
         <f>IF(AND(BC16="",BD16=""),"",IF(OR(BC16="",BD16=""),"불일치",IF(ABS(BC16-BD16)&lt;=MAX(1,ABS(BD16))*1E-9,"일치","불일치")))</f>
@@ -12779,7 +12779,7 @@
         <v/>
       </c>
       <c r="BM16" t="n">
-        <v>27345644055</v>
+        <v>27062873035</v>
       </c>
       <c r="BN16">
         <f>IF(AND(BL16="",BM16=""),"",IF(OR(BL16="",BM16=""),"불일치",IF(ABS(BL16-BM16)&lt;=MAX(1,ABS(BM16))*1E-9,"일치","불일치")))</f>
@@ -12790,7 +12790,7 @@
         <v/>
       </c>
       <c r="BP16" t="n">
-        <v>-0.07494893595769068</v>
+        <v>-0.07573205262979205</v>
       </c>
       <c r="BQ16">
         <f>IF(AND(BO16="",BP16=""),"",IF(OR(BO16="",BP16=""),"불일치",IF(ABS(BO16-BP16)&lt;=MAX(1,ABS(BP16))*1E-9,"일치","불일치")))</f>
@@ -13076,7 +13076,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>21104400000</v>
+        <v>20531800000</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>2985511589</v>
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="BA18" t="n">
-        <v>0.08759842606281154</v>
+        <v>0.09004141005659513</v>
       </c>
       <c r="BB18">
         <f>IF(AND(AZ18="",BA18=""),"",IF(OR(AZ18="",BA18=""),"불일치",IF(ABS(AZ18-BA18)&lt;=MAX(1,ABS(BA18))*1E-9,"일치","불일치")))</f>
@@ -13244,7 +13244,7 @@
         <v/>
       </c>
       <c r="BD18" t="n">
-        <v>2.318768218286234</v>
+        <v>2.383435061027285</v>
       </c>
       <c r="BE18">
         <f>IF(AND(BC18="",BD18=""),"",IF(OR(BC18="",BD18=""),"불일치",IF(ABS(BC18-BD18)&lt;=MAX(1,ABS(BD18))*1E-9,"일치","불일치")))</f>
@@ -13277,7 +13277,7 @@
         <v/>
       </c>
       <c r="BM18" t="n">
-        <v>13712195291</v>
+        <v>13139595291</v>
       </c>
       <c r="BN18">
         <f>IF(AND(BL18="",BM18=""),"",IF(OR(BL18="",BM18=""),"불일치",IF(ABS(BL18-BM18)&lt;=MAX(1,ABS(BM18))*1E-9,"일치","불일치")))</f>
@@ -13288,7 +13288,7 @@
         <v/>
       </c>
       <c r="BP18" t="n">
-        <v>-0.07454364507708644</v>
+        <v>-0.07779212345300537</v>
       </c>
       <c r="BQ18">
         <f>IF(AND(BO18="",BP18=""),"",IF(OR(BO18="",BP18=""),"불일치",IF(ABS(BO18-BP18)&lt;=MAX(1,ABS(BP18))*1E-9,"일치","불일치")))</f>
@@ -13328,7 +13328,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>41509711380</v>
+        <v>40156133835</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-17872159378</v>
@@ -13485,7 +13485,7 @@
         <v/>
       </c>
       <c r="BA19" t="n">
-        <v>-1.886205520950071</v>
+        <v>-1.949785482330411</v>
       </c>
       <c r="BB19">
         <f>IF(AND(AZ19="",BA19=""),"",IF(OR(AZ19="",BA19=""),"불일치",IF(ABS(AZ19-BA19)&lt;=MAX(1,ABS(BA19))*1E-9,"일치","불일치")))</f>
@@ -13496,7 +13496,7 @@
         <v/>
       </c>
       <c r="BD19" t="n">
-        <v>4.679373912813749</v>
+        <v>4.837105617740055</v>
       </c>
       <c r="BE19">
         <f>IF(AND(BC19="",BD19=""),"",IF(OR(BC19="",BD19=""),"불일치",IF(ABS(BC19-BD19)&lt;=MAX(1,ABS(BD19))*1E-9,"일치","불일치")))</f>
@@ -13529,7 +13529,7 @@
         <v/>
       </c>
       <c r="BM19" t="n">
-        <v>209032794435</v>
+        <v>207679216890</v>
       </c>
       <c r="BN19">
         <f>IF(AND(BL19="",BM19=""),"",IF(OR(BL19="",BM19=""),"불일치",IF(ABS(BL19-BM19)&lt;=MAX(1,ABS(BM19))*1E-9,"일치","불일치")))</f>
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="BP19" t="n">
-        <v>-0.276224615247894</v>
+        <v>-0.2780249467503662</v>
       </c>
       <c r="BQ19">
         <f>IF(AND(BO19="",BP19=""),"",IF(OR(BO19="",BP19=""),"불일치",IF(ABS(BO19-BP19)&lt;=MAX(1,ABS(BP19))*1E-9,"일치","불일치")))</f>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>53744640620</v>
+        <v>52586133840</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>14255757950</v>
@@ -13734,7 +13734,7 @@
         <v/>
       </c>
       <c r="BA20" t="n">
-        <v>-0.8593265061635461</v>
+        <v>-0.8782580288089116</v>
       </c>
       <c r="BB20">
         <f>IF(AND(AZ20="",BA20=""),"",IF(OR(AZ20="",BA20=""),"불일치",IF(ABS(AZ20-BA20)&lt;=MAX(1,ABS(BA20))*1E-9,"일치","불일치")))</f>
@@ -13745,7 +13745,7 @@
         <v/>
       </c>
       <c r="BD20" t="n">
-        <v>6.742371203951312</v>
+        <v>6.890910033157136</v>
       </c>
       <c r="BE20">
         <f>IF(AND(BC20="",BD20=""),"",IF(OR(BC20="",BD20=""),"불일치",IF(ABS(BC20-BD20)&lt;=MAX(1,ABS(BD20))*1E-9,"일치","불일치")))</f>
@@ -13778,7 +13778,7 @@
         <v/>
       </c>
       <c r="BM20" t="n">
-        <v>660723520379</v>
+        <v>659565013599</v>
       </c>
       <c r="BN20">
         <f>IF(AND(BL20="",BM20=""),"",IF(OR(BL20="",BM20=""),"불일치",IF(ABS(BL20-BM20)&lt;=MAX(1,ABS(BM20))*1E-9,"일치","불일치")))</f>
@@ -13789,7 +13789,7 @@
         <v/>
       </c>
       <c r="BP20" t="n">
-        <v>0.088425315852971</v>
+        <v>0.08858063235070385</v>
       </c>
       <c r="BQ20">
         <f>IF(AND(BO20="",BP20=""),"",IF(OR(BO20="",BP20=""),"불일치",IF(ABS(BO20-BP20)&lt;=MAX(1,ABS(BP20))*1E-9,"일치","불일치")))</f>
@@ -13826,7 +13826,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>21430753080</v>
+        <v>21834414525</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-3443498622</v>
@@ -13983,7 +13983,7 @@
         <v/>
       </c>
       <c r="BA21" t="n">
-        <v>-0.1523446733678666</v>
+        <v>-0.1495282172215699</v>
       </c>
       <c r="BB21">
         <f>IF(AND(AZ21="",BA21=""),"",IF(OR(AZ21="",BA21=""),"불일치",IF(ABS(AZ21-BA21)&lt;=MAX(1,ABS(BA21))*1E-9,"일치","불일치")))</f>
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="BD21" t="n">
-        <v>1.452620144415382</v>
+        <v>1.425764982081653</v>
       </c>
       <c r="BE21">
         <f>IF(AND(BC21="",BD21=""),"",IF(OR(BC21="",BD21=""),"불일치",IF(ABS(BC21-BD21)&lt;=MAX(1,ABS(BD21))*1E-9,"일치","불일치")))</f>
@@ -14027,7 +14027,7 @@
         <v/>
       </c>
       <c r="BM21" t="n">
-        <v>28560571778</v>
+        <v>28964233223</v>
       </c>
       <c r="BN21">
         <f>IF(AND(BL21="",BM21=""),"",IF(OR(BL21="",BM21=""),"불일치",IF(ABS(BL21-BM21)&lt;=MAX(1,ABS(BM21))*1E-9,"일치","불일치")))</f>
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="BP21" t="n">
-        <v>-0.1355318283922348</v>
+        <v>-0.133642982474199</v>
       </c>
       <c r="BQ21">
         <f>IF(AND(BO21="",BP21=""),"",IF(OR(BO21="",BP21=""),"불일치",IF(ABS(BO21-BP21)&lt;=MAX(1,ABS(BP21))*1E-9,"일치","불일치")))</f>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>73568114880</v>
+        <v>67791131500</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-1424637813</v>
@@ -14232,7 +14232,7 @@
         <v/>
       </c>
       <c r="BA22" t="n">
-        <v>-0.02748059187458685</v>
+        <v>-0.0298224162256386</v>
       </c>
       <c r="BB22">
         <f>IF(AND(AZ22="",BA22=""),"",IF(OR(AZ22="",BA22=""),"불일치",IF(ABS(AZ22-BA22)&lt;=MAX(1,ABS(BA22))*1E-9,"일치","불일치")))</f>
@@ -14243,7 +14243,7 @@
         <v/>
       </c>
       <c r="BD22" t="n">
-        <v>0.6292491661708323</v>
+        <v>0.6828721385923467</v>
       </c>
       <c r="BE22">
         <f>IF(AND(BC22="",BD22=""),"",IF(OR(BC22="",BD22=""),"불일치",IF(ABS(BC22-BD22)&lt;=MAX(1,ABS(BD22))*1E-9,"일치","불일치")))</f>
@@ -14276,7 +14276,7 @@
         <v/>
       </c>
       <c r="BM22" t="n">
-        <v>106186891768</v>
+        <v>100409908388</v>
       </c>
       <c r="BN22">
         <f>IF(AND(BL22="",BM22=""),"",IF(OR(BL22="",BM22=""),"불일치",IF(ABS(BL22-BM22)&lt;=MAX(1,ABS(BM22))*1E-9,"일치","불일치")))</f>
@@ -14287,7 +14287,7 @@
         <v/>
       </c>
       <c r="BP22" t="n">
-        <v>0.01518765230009308</v>
+        <v>0.01606145864378398</v>
       </c>
       <c r="BQ22">
         <f>IF(AND(BO22="",BP22=""),"",IF(OR(BO22="",BP22=""),"불일치",IF(ABS(BO22-BP22)&lt;=MAX(1,ABS(BP22))*1E-9,"일치","불일치")))</f>
@@ -14324,7 +14324,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>34003001637</v>
+        <v>31429894860</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-2497579973</v>
@@ -14481,7 +14481,7 @@
         <v/>
       </c>
       <c r="BA23" t="n">
-        <v>-0.02784500351197627</v>
+        <v>-0.03012462193136334</v>
       </c>
       <c r="BB23">
         <f>IF(AND(AZ23="",BA23=""),"",IF(OR(AZ23="",BA23=""),"불일치",IF(ABS(AZ23-BA23)&lt;=MAX(1,ABS(BA23))*1E-9,"일치","불일치")))</f>
@@ -14492,7 +14492,7 @@
         <v/>
       </c>
       <c r="BD23" t="n">
-        <v>1.628932904668319</v>
+        <v>1.762290598512044</v>
       </c>
       <c r="BE23">
         <f>IF(AND(BC23="",BD23=""),"",IF(OR(BC23="",BD23=""),"불일치",IF(ABS(BC23-BD23)&lt;=MAX(1,ABS(BD23))*1E-9,"일치","불일치")))</f>
@@ -14525,7 +14525,7 @@
         <v/>
       </c>
       <c r="BM23" t="n">
-        <v>32413541218</v>
+        <v>29840434441</v>
       </c>
       <c r="BN23">
         <f>IF(AND(BL23="",BM23=""),"",IF(OR(BL23="",BM23=""),"불일치",IF(ABS(BL23-BM23)&lt;=MAX(1,ABS(BM23))*1E-9,"일치","불일치")))</f>
@@ -14536,7 +14536,7 @@
         <v/>
       </c>
       <c r="BP23" t="n">
-        <v>-0.04941514144435806</v>
+        <v>-0.05367615297849946</v>
       </c>
       <c r="BQ23">
         <f>IF(AND(BO23="",BP23=""),"",IF(OR(BO23="",BP23=""),"불일치",IF(ABS(BO23-BP23)&lt;=MAX(1,ABS(BP23))*1E-9,"일치","불일치")))</f>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>492910902000</v>
+        <v>495008395200</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>9593627586</v>
@@ -14730,7 +14730,7 @@
         <v/>
       </c>
       <c r="BA24" t="n">
-        <v>0.03192285079342798</v>
+        <v>0.03178758447650668</v>
       </c>
       <c r="BB24">
         <f>IF(AND(AZ24="",BA24=""),"",IF(OR(AZ24="",BA24=""),"불일치",IF(ABS(AZ24-BA24)&lt;=MAX(1,ABS(BA24))*1E-9,"일치","불일치")))</f>
@@ -14741,7 +14741,7 @@
         <v/>
       </c>
       <c r="BD24" t="n">
-        <v>0.6293774261986196</v>
+        <v>0.626710572697778</v>
       </c>
       <c r="BE24">
         <f>IF(AND(BC24="",BD24=""),"",IF(OR(BC24="",BD24=""),"불일치",IF(ABS(BC24-BD24)&lt;=MAX(1,ABS(BD24))*1E-9,"일치","불일치")))</f>
@@ -14774,7 +14774,7 @@
         <v/>
       </c>
       <c r="BM24" t="n">
-        <v>556341483300</v>
+        <v>558438976500</v>
       </c>
       <c r="BN24">
         <f>IF(AND(BL24="",BM24=""),"",IF(OR(BL24="",BM24=""),"불일치",IF(ABS(BL24-BM24)&lt;=MAX(1,ABS(BM24))*1E-9,"일치","불일치")))</f>
@@ -14785,7 +14785,7 @@
         <v/>
       </c>
       <c r="BP24" t="n">
-        <v>0.027739505369004</v>
+        <v>0.02763531596544999</v>
       </c>
       <c r="BQ24">
         <f>IF(AND(BO24="",BP24=""),"",IF(OR(BO24="",BP24=""),"불일치",IF(ABS(BO24-BP24)&lt;=MAX(1,ABS(BP24))*1E-9,"일치","불일치")))</f>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>101645669160</v>
+        <v>99286803420</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>9185573010</v>
@@ -14982,7 +14982,7 @@
         <v/>
       </c>
       <c r="BA25" t="n">
-        <v>-0.18564971941201</v>
+        <v>-0.1900604038904811</v>
       </c>
       <c r="BB25">
         <f>IF(AND(AZ25="",BA25=""),"",IF(OR(AZ25="",BA25=""),"불일치",IF(ABS(AZ25-BA25)&lt;=MAX(1,ABS(BA25))*1E-9,"일치","불일치")))</f>
@@ -14993,7 +14993,7 @@
         <v/>
       </c>
       <c r="BD25" t="n">
-        <v>2.746237335656692</v>
+        <v>2.811482715121538</v>
       </c>
       <c r="BE25">
         <f>IF(AND(BC25="",BD25=""),"",IF(OR(BC25="",BD25=""),"불일치",IF(ABS(BC25-BD25)&lt;=MAX(1,ABS(BD25))*1E-9,"일치","불일치")))</f>
@@ -15026,7 +15026,7 @@
         <v/>
       </c>
       <c r="BM25" t="n">
-        <v>149044621538</v>
+        <v>146685755798</v>
       </c>
       <c r="BN25">
         <f>IF(AND(BL25="",BM25=""),"",IF(OR(BL25="",BM25=""),"불일치",IF(ABS(BL25-BM25)&lt;=MAX(1,ABS(BM25))*1E-9,"일치","불일치")))</f>
@@ -15037,7 +15037,7 @@
         <v/>
       </c>
       <c r="BP25" t="n">
-        <v>0.2943156366418496</v>
+        <v>0.2990485506745986</v>
       </c>
       <c r="BQ25">
         <f>IF(AND(BO25="",BP25=""),"",IF(OR(BO25="",BP25=""),"불일치",IF(ABS(BO25-BP25)&lt;=MAX(1,ABS(BP25))*1E-9,"일치","불일치")))</f>
@@ -15074,7 +15074,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20474803320</v>
+        <v>20866041600</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>2165012133</v>
@@ -15231,7 +15231,7 @@
         <v/>
       </c>
       <c r="BA26" t="n">
-        <v>0.02806027555042712</v>
+        <v>0.02753414538385661</v>
       </c>
       <c r="BB26">
         <f>IF(AND(AZ26="",BA26=""),"",IF(OR(AZ26="",BA26=""),"불일치",IF(ABS(AZ26-BA26)&lt;=MAX(1,ABS(BA26))*1E-9,"일치","불일치")))</f>
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="BD26" t="n">
-        <v>2.17451278501463</v>
+        <v>2.133740670295606</v>
       </c>
       <c r="BE26">
         <f>IF(AND(BC26="",BD26=""),"",IF(OR(BC26="",BD26=""),"불일치",IF(ABS(BC26-BD26)&lt;=MAX(1,ABS(BD26))*1E-9,"일치","불일치")))</f>
@@ -15275,7 +15275,7 @@
         <v/>
       </c>
       <c r="BM26" t="n">
-        <v>42433996732</v>
+        <v>42825235012</v>
       </c>
       <c r="BN26">
         <f>IF(AND(BL26="",BM26=""),"",IF(OR(BL26="",BM26=""),"불일치",IF(ABS(BL26-BM26)&lt;=MAX(1,ABS(BM26))*1E-9,"일치","불일치")))</f>
@@ -15286,7 +15286,7 @@
         <v/>
       </c>
       <c r="BP26" t="n">
-        <v>0.02899666476790075</v>
+        <v>0.02873176008620195</v>
       </c>
       <c r="BQ26">
         <f>IF(AND(BO26="",BP26=""),"",IF(OR(BO26="",BP26=""),"불일치",IF(ABS(BO26-BP26)&lt;=MAX(1,ABS(BP26))*1E-9,"일치","불일치")))</f>

</xml_diff>